<commit_message>
fix: 修正文档om rest, create domain的样例
git-svn-id: http://192.168.20.11/sequoiadb/trunk@27632 6121f079-4a18-41d3-8c30-8870a322f2c2
</commit_message>
<xml_diff>
--- a/internal_doc/03.开发设计/OM/om_sequoiadb_operation.xlsx
+++ b/internal_doc/03.开发设计/OM/om_sequoiadb_operation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26670" windowHeight="11910" activeTab="1"/>
+    <workbookView windowWidth="28695" windowHeight="13050" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="1" r:id="rId1"/>
@@ -29,11 +29,10 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t xml:space="preserve">Author:
+          <t>Author:
 增加flag，数字和字符串两种格式
 后续版本新增的命令，参数名采用括号内名字。逐渐替换掉旧的名字</t>
         </r>
@@ -44,11 +43,10 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t xml:space="preserve">Author:
+          <t>Author:
 可以暂时不支持多条</t>
         </r>
       </text>
@@ -58,11 +56,10 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t xml:space="preserve">Author:
+          <t>Author:
 sort-》orderby
 增加flag，下同
 兼容处理</t>
@@ -74,11 +71,10 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t xml:space="preserve">Author:
+          <t>Author:
 增加flag</t>
         </r>
       </text>
@@ -88,7 +84,6 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
@@ -103,11 +98,10 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t xml:space="preserve">Author:
+          <t>Author:
 需要直连数据节点！</t>
         </r>
       </text>
@@ -117,11 +111,10 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t xml:space="preserve">Author:
+          <t>Author:
 归到 list collectionspaces domain做为参数</t>
         </r>
       </text>
@@ -131,11 +124,10 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t xml:space="preserve">Author:
+          <t>Author:
 isasync -》 flag</t>
         </r>
       </text>
@@ -1215,7 +1207,7 @@
 options：设置其他属性</t>
   </si>
   <si>
-    <t>cmd=create domain&amp;options={"AutoSplit":true,{"Groups":["g1","g2"]}}</t>
+    <t>cmd=create domain&amp;options={"AutoSplit":true,"Groups":["g1","g2"]}</t>
   </si>
   <si>
     <t>create group</t>
@@ -1589,11 +1581,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1615,8 +1607,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1629,9 +1622,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1639,15 +1631,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1662,17 +1646,53 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1683,8 +1703,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1699,68 +1744,8 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1848,13 +1833,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1872,25 +1857,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1908,7 +1875,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1926,7 +1929,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1938,31 +1959,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1974,19 +1995,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1998,31 +2007,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2077,17 +2062,61 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
       </top>
       <bottom style="double">
-        <color rgb="FF3F3F3F"/>
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2096,7 +2125,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4"/>
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2116,61 +2145,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
       </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
       </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2182,10 +2167,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2194,138 +2179,138 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
@@ -2408,9 +2393,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2467,6 +2449,7 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
     <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2"/>
 </styleSheet>
 </file>
 
@@ -2768,7 +2751,7 @@
       </c>
     </row>
     <row r="2" ht="27" spans="1:1">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="40" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4365,7 +4348,7 @@
       <c r="F68" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="G68" s="40" t="s">
+      <c r="G68" s="32" t="s">
         <v>246</v>
       </c>
       <c r="H68" s="32" t="s">

</xml_diff>